<commit_message>
Add sea level curves plot
</commit_message>
<xml_diff>
--- a/ISMIP7/tier2/configs/variations.xlsx
+++ b/ISMIP7/tier2/configs/variations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Beren017/Documents/GitHub/contrib-ismip/ISMIP7/tier2/configs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBC4EE8B-BEF8-4440-8828-6791376E00EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8291DA-67EF-DB47-A321-B21E9930EE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19320" xr2:uid="{5B6D99C4-B9F7-914C-8B64-12AA687BA3A6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="47">
   <si>
     <t>Forcing variations</t>
   </si>
@@ -98,32 +98,104 @@
     <t>Thermodynamics: constant</t>
   </si>
   <si>
-    <t>m009</t>
-  </si>
-  <si>
-    <t>m010</t>
-  </si>
-  <si>
     <t>GIA: uniform fast relaxation time 3000 yr</t>
   </si>
   <si>
     <t>GIA: uniform slow relaxation time 200 yr</t>
   </si>
   <si>
-    <t>Calving: threshold thickness 100 m</t>
-  </si>
-  <si>
-    <t>Calving: threshold thickness 200 m</t>
+    <t>Simulation</t>
+  </si>
+  <si>
+    <t>Forcing variation</t>
+  </si>
+  <si>
+    <t>Model variation</t>
+  </si>
+  <si>
+    <t>P001</t>
+  </si>
+  <si>
+    <t>P002</t>
+  </si>
+  <si>
+    <t>P003</t>
+  </si>
+  <si>
+    <t>P004</t>
+  </si>
+  <si>
+    <t>P005</t>
+  </si>
+  <si>
+    <t>P006</t>
+  </si>
+  <si>
+    <t>P007</t>
+  </si>
+  <si>
+    <t>P008</t>
+  </si>
+  <si>
+    <t>P009</t>
+  </si>
+  <si>
+    <t>P010</t>
+  </si>
+  <si>
+    <t>P011</t>
+  </si>
+  <si>
+    <t>P012</t>
+  </si>
+  <si>
+    <t>P013</t>
+  </si>
+  <si>
+    <t>P014</t>
+  </si>
+  <si>
+    <t>P015</t>
+  </si>
+  <si>
+    <t>P016</t>
+  </si>
+  <si>
+    <t>P017</t>
+  </si>
+  <si>
+    <t>P018</t>
+  </si>
+  <si>
+    <t>P019</t>
+  </si>
+  <si>
+    <t>P020</t>
+  </si>
+  <si>
+    <t>Base experiment</t>
+  </si>
+  <si>
+    <t>C001</t>
+  </si>
+  <si>
+    <t>C007</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -485,18 +557,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35E1B1AD-E51E-D34F-B490-07230D53272C}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="31" customWidth="1"/>
+    <col min="2" max="2" width="16.5" customWidth="1"/>
+    <col min="3" max="3" width="16.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -504,7 +577,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -512,12 +585,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -525,23 +598,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -549,7 +622,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -557,7 +630,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -565,7 +638,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -573,7 +646,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -581,23 +654,302 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>24</v>
       </c>
+      <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" t="s">
+        <v>3</v>
+      </c>
+      <c r="D18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" t="s">
+        <v>1</v>
+      </c>
+      <c r="D22" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1</v>
+      </c>
+      <c r="D23" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1</v>
+      </c>
+      <c r="D24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1</v>
+      </c>
+      <c r="D25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>35</v>
+      </c>
+      <c r="B27" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" t="s">
+        <v>45</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1</v>
+      </c>
+      <c r="D28" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>37</v>
+      </c>
+      <c r="B29" t="s">
+        <v>46</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1</v>
+      </c>
+      <c r="D29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1</v>
+      </c>
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>39</v>
+      </c>
+      <c r="B31" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1</v>
+      </c>
+      <c r="D31" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" t="s">
+        <v>45</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1</v>
+      </c>
+      <c r="D32" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>41</v>
+      </c>
+      <c r="B33" t="s">
+        <v>46</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1</v>
+      </c>
+      <c r="D33" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" t="s">
+        <v>45</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1</v>
+      </c>
+      <c r="D34" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>43</v>
+      </c>
+      <c r="B35" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1</v>
+      </c>
+      <c r="D35" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>